<commit_message>
copy: fase percobaan — pricing jadi gratis masa uji (Rp0 + harga coret), hapus 'Beli via QRIS — Segera'; tracker: keputusan infra Cloudflare+Supabase, payment ditunda
</commit_message>
<xml_diff>
--- a/download/Issue_Tracker_Sayangin.xlsx
+++ b/download/Issue_Tracker_Sayangin.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="206">
   <si>
     <t xml:space="preserve">Issue Tracker — Sayangin (15 isu, siap dieksekusi)</t>
   </si>
@@ -109,13 +109,13 @@
     <t xml:space="preserve">S-03</t>
   </si>
   <si>
-    <t xml:space="preserve">Belum ada keputusan arsitektur deploy</t>
+    <t xml:space="preserve">Keputusan deploy: Cloudflare + Supabase ✅ (diputuskan 31 Okt)</t>
   </si>
   <si>
     <t xml:space="preserve">SQLite file + rate-limit in-memory tidak survivable di serverless/restart; app baru jalan di localhost</t>
   </si>
   <si>
-    <t xml:space="preserve">Pilih jalur (lihat sheet 'Keputusan Infra'): A) VPS/Railway + SQLite + Litestream, atau B) Vercel + Turso + Upstash; lalu deploy + pasang domain</t>
+    <t xml:space="preserve">PILIHAN USER: Cloudflare (Pages/Workers via @opennextjs/cloudflare, nodejs_compat) + Supabase Postgres. Migrasi: provider Prisma sqlite → postgresql, koneksi via pooler (port 6543), prisma migrate dari nol</t>
   </si>
   <si>
     <t xml:space="preserve">App hidup di domain produksi dengan DB persisten; satu deploy penuh sukses dari repo</t>
@@ -130,10 +130,10 @@
     <t xml:space="preserve">src/lib/rate-limit.ts pakai Map per-proses — limit gugur saat restart/deploy, bisa di-bypass spam</t>
   </si>
   <si>
-    <t xml:space="preserve">Ikut jalur S-03: jalur A → pindah bucket ke tabel SQLite (atau tetap in-memory + dokumentasi karena 1 instance), jalur B → Upstash Redis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restart server → counter limit tidak reset; ujung-ke-ujung: spam 6x confess kena 429</t>
+    <t xml:space="preserve">Di Cloudflare: Upstash Redis (paling gampang, API tinggal diganti) atau Durable Objects. Hindari KV — eventual consistency kurang cocok untuk counter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restart/redeploy → counter limit tidak reset; ujung-ke-ujung: spam 6x confess kena 429</t>
   </si>
   <si>
     <t xml:space="preserve">S-05</t>
@@ -145,7 +145,7 @@
     <t xml:space="preserve">DB berisi surat yang emosional tapi tidak ada backup; error produksi tidak terpantau (tidak ada Sentry)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jalur A: Litestream → object storage. Jalur B: backup bawaan Turso. Pasang Sentry free tier (source maps on)</t>
+    <t xml:space="preserve">Supabase free tier tidak ada auto-backup → cron GitHub Actions pg_dump mingguan ke storage; Sentry free tier (source maps on)</t>
   </si>
   <si>
     <t xml:space="preserve">Restore drill 1x sukses dari backup; error test muncul di Sentry &lt; 1 menit</t>
@@ -271,51 +271,57 @@
     <t xml:space="preserve">S-12</t>
   </si>
   <si>
+    <t xml:space="preserve">P3 — ditunda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nanti — setelah fase percobaan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment QRIS ditunda sampai fase percobaan validasi ✅ (keputusan 31 Okt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase sekarang = uji minat pasar; semua kado gratis. Copy sudah diganti jadi 'gratis selama masa uji' (Pricing, FAQ, Hero, metadata)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kalau nanti sinyal bagus: Midtrans Snap (QRIS friendly) — order per kado, webhook verifikasi, flag isPaid + paidAt di model Gift; kado terkunci sampai terbayar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alur sandbox Midtrans: bayar → webhook → kado terbuka; signature invalid ditolak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merata — 4 fase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kualitas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nol test, nol CI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tidak ada file *.test.* di repo; API kritis (confess, reply, redeem) tidak terlindungi regresi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitest untuk lib kritis (moderation, rate-limit, token, gift-data) + Playwright e2e 3 jalur: buat confess → buka → balas; GitHub Actions lint+test tiap push</t>
+  </si>
+  <si>
+    <t xml:space="preserve">npm test hijau; Actions merah kalau ada regresi di jalur confess</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S-14</t>
+  </si>
+  <si>
     <t xml:space="preserve">P3</t>
   </si>
   <si>
     <t xml:space="preserve">3 — Monetisasi</t>
   </si>
   <si>
-    <t xml:space="preserve">Revenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Copy menyebut 'sekali bayar' tapi payment belum ada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metadata OG menjanjikan kado berbayar; grep midtrans/xendit/stripe = 0 hasil di src/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Midtrans Snap (QRIS friendly): order per kado, webhook verifikasi tanda tangan, flag isPaid + paidAt di model Gift; kado terkunci sampai terbayar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alur sandbox Midtrans: bayar → webhook → kado terbuka; signature invalid ditolak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Merata — 4 fase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kualitas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nol test, nol CI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tidak ada file *.test.* di repo; API kritis (confess, reply, redeem) tidak terlindungi regresi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vitest untuk lib kritis (moderation, rate-limit, token, gift-data) + Playwright e2e 3 jalur: buat confess → buka → balas; GitHub Actions lint+test tiap push</t>
-  </si>
-  <si>
-    <t xml:space="preserve">npm test hijau; Actions merah kalau ada regresi di jalur confess</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S-14</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dependencies bloat</t>
   </si>
   <si>
@@ -397,7 +403,7 @@
     <t xml:space="preserve">1–2</t>
   </si>
   <si>
-    <t xml:space="preserve">AMBIL KEPUTUSAN deploy (sheet 3): setup hosting + DB persisten + domain</t>
+    <t xml:space="preserve">Setup Cloudflare (adapter OpenNext) + Supabase Postgres + domain — keputusan final 31 Okt</t>
   </si>
   <si>
     <t xml:space="preserve">GERBANG 1 — app hidup di produksi</t>
@@ -406,7 +412,7 @@
     <t xml:space="preserve">3</t>
   </si>
   <si>
-    <t xml:space="preserve">Rate limiter ikut jalur yang dipilih (Redis / SQLite-backed)</t>
+    <t xml:space="preserve">Rate limiter pindah ke Upstash Redis (atau Durable Objects)</t>
   </si>
   <si>
     <t xml:space="preserve">Anti-spam survivable restart</t>
@@ -526,94 +532,118 @@
     <t xml:space="preserve">Kalau waktu mepet: Jalur A dipilih + milestone 1–2 saja sudah membuat Sayangin 10x lebih layak pakai.</t>
   </si>
   <si>
-    <t xml:space="preserve">Keputusan Infra — pilih SATU jalur sebelum gerbang 1 (S-03)</t>
+    <t xml:space="preserve">Keputusan Infra — DIPUTUSKAN 31 Okt 2026: Cloudflare + Supabase (S-03 ✅)</t>
   </si>
   <si>
     <t xml:space="preserve">Aspek</t>
   </si>
   <si>
+    <t xml:space="preserve">Keputusan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detail / langkah setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hosting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloudflare Pages/Workers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adapter @opennextjs/cloudflare + nodejs_compat di wrangler.toml; domain mengarah ke Cloudflare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Database</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supabase Postgres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">schema.prisma: provider "postgresql"; DATABASE_URL = pooler Supabase (port 6543, transaction mode) — cocok untuk serverless</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migrasi DB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prisma migrate dari nol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data SQLite lama (db/custom.db) hanya data uji — tidak dibawa; jalankan db:generate + migrate deploy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upstash Redis (atau Durable Objects)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API rate-limit.ts tinggal diganti di dalamnya; hindari Cloudflare KV — eventual consistency tidak cocok untuk counter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub Actions cron → pg_dump mingguan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supabase free tier tidak ada auto-backup; dump → Cloudflare R2 / storage lain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitoring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sentry free tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasang setelah deploy (S-05); error produksi langsung terpantau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biaya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$0 — keduanya free tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naik hanya kalau traffic ramai; tier gratis Supabase cukup untuk fase percobaan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✔ FINAL — payment QRIS ditunda sampai fase percobaan validasi (S-12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lanjut ke S-04 (rate limit) &amp; S-05 (backup) dengan stack ini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referensi — dua jalur lain yang tidak dipilih (kalau nanti butuh pindah):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jalur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kekuatan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kenapa tidak sekarang</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jalur A — VPS/Railway + SQLite + Litestream</t>
   </si>
   <si>
+    <t xml:space="preserve">Paling cepat ke produksi; schema SQLite tidak berubah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Butuh kelola server sendiri; Cloudflare+Supabase sudah dipilih dan free tier</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jalur B — Vercel + Turso + Upstash</t>
   </si>
   <si>
-    <t xml:space="preserve">Biaya bulanan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈ $5–10 (VPS murah) atau ~$5 Railway</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$0 di tier gratis (perkiraan; naik kalau traffic ramai)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usaha migrasi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimal — schema SQLite tetap, tinggal deploy + pasang Litestream</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sedang — ganti provider Prisma ke libsql, ubah rate-limit ke Redis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Litestream → object storage (S3/Cloudflare R2), wajib dipasang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bawaan Turso (point-in-time restore)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rate limit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In-memory cukup — 1 instance, restart jarang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wajib pindah ke Upstash Redis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upront kerja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">± 1 hari ke produksi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">± 2–3 hari (dua layanan baru diintegrasikan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cocok jika</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mau online minggu ini, hemat, skala komunitas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mau zero-ops dan siap tumbuh tanpa pikir server</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risiko utama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Satu server = satu titik gagal; butuh disiplin backup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cold start + ketergantungan 2 vendor; integrasi butuh test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rekomendasi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">✔ PILIH JALUR A dulu — cepat ke produksi tanpa migrasi kode besar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Simpan sebagai target pindah saat traffic &gt; ± 100 rb view/bulan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catatan teknis jalur B: di schema.prisma ganti provider ke "libsql" + DATABASE_URL ke Turso; rate-limit.ts pindah bucket ke Redis (API sama).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jalur A wajib: litestream.yml (replicate ke R2) sebagai systemd service — backup diverifikasi lewat restore drill S-05.</t>
+    <t xml:space="preserve">Zero-ops serverless; Turso SQLite-compatible (migrasi paling gampang)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User memilih Postgres Supabase + Cloudflare; struktur tetap tersimpan sebagai referensi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urutan kerja tetap: S-01 (crypto) → S-02 (migrate) → setup stack ini (S-03) → S-04 → S-05 = Milestone 1 'Aman dipromosikan'.</t>
   </si>
 </sst>
 </file>
@@ -767,7 +797,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -866,6 +896,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1274,7 +1308,7 @@
       </c>
       <c r="K6" s="10"/>
     </row>
-    <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="5" t="s">
         <v>26</v>
       </c>
@@ -1304,7 +1338,7 @@
       </c>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="9" t="s">
         <v>31</v>
       </c>
@@ -1334,7 +1368,7 @@
       </c>
       <c r="K8" s="10"/>
     </row>
-    <row r="9" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
         <v>36</v>
       </c>
@@ -1544,7 +1578,7 @@
       </c>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="9" t="s">
         <v>80</v>
       </c>
@@ -1609,64 +1643,64 @@
         <v>95</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>90</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I18" s="12" t="n">
         <v>0.5</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>90</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I19" s="8" t="n">
         <v>0.5</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
@@ -1674,7 +1708,7 @@
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="H20" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I20" s="14" t="n">
         <f aca="false">SUM(I5:I19)</f>
@@ -1685,7 +1719,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1728,7 +1762,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -1738,27 +1772,27 @@
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1766,19 +1800,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D5" s="16" t="s">
         <v>12</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1786,36 +1820,36 @@
         <v>2</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>20</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F6" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="G6" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G6" s="19" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>26</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G7" s="16" t="s">
         <v>20</v>
@@ -1826,16 +1860,16 @@
         <v>4</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>31</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>26</v>
@@ -1846,16 +1880,16 @@
         <v>5</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>36</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G9" s="16" t="s">
         <v>26</v>
@@ -1863,7 +1897,7 @@
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="21" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C10" s="21"/>
       <c r="D10" s="21"/>
@@ -1876,16 +1910,16 @@
         <v>6</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D11" s="19" t="s">
         <v>41</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G11" s="19" t="s">
         <v>26</v>
@@ -1896,19 +1930,19 @@
         <v>7</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D12" s="16" t="s">
         <v>49</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1916,16 +1950,16 @@
         <v>8</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D13" s="19" t="s">
         <v>55</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G13" s="19" t="s">
         <v>26</v>
@@ -1933,7 +1967,7 @@
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C14" s="21"/>
       <c r="D14" s="21"/>
@@ -1946,19 +1980,19 @@
         <v>9</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>61</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1966,19 +2000,19 @@
         <v>10</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D16" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1986,16 +2020,16 @@
         <v>11</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>74</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G17" s="16" t="s">
         <v>26</v>
@@ -2003,7 +2037,7 @@
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="21" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C18" s="21"/>
       <c r="D18" s="21"/>
@@ -2016,19 +2050,19 @@
         <v>12</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D19" s="19" t="s">
         <v>88</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2036,16 +2070,16 @@
         <v>13</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D20" s="16" t="s">
         <v>80</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G20" s="16" t="s">
         <v>74</v>
@@ -2056,19 +2090,19 @@
         <v>14</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D21" s="19" t="s">
         <v>95</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2076,24 +2110,24 @@
         <v>15</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="21" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C23" s="21"/>
       <c r="D23" s="21"/>
@@ -2103,12 +2137,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -2134,7 +2168,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:D15"/>
+  <dimension ref="B2:D19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
@@ -2144,7 +2178,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2152,111 +2186,144 @@
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="22" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="23" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="22" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="23" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="22" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="23" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="24" t="s">
-        <v>191</v>
+        <v>11</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="3" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="3" t="s">
+    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="25" t="s">
         <v>195</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="22" t="s">
+        <v>199</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="3" t="s">
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
security+db: S-01 slug & senderKey pakai CSPRNG (crypto.getRandomValues, siap Cloudflare), hapus duplikat generator di confess route; S-02 baseline prisma migrate + hapus script db:push --accept-data-loss
</commit_message>
<xml_diff>
--- a/download/Issue_Tracker_Sayangin.xlsx
+++ b/download/Issue_Tracker_Sayangin.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="208">
   <si>
     <t xml:space="preserve">Issue Tracker — Sayangin (15 isu, siap dieksekusi)</t>
   </si>
@@ -88,6 +88,9 @@
     <t xml:space="preserve">grep Math.random() di jalur token/slug = 0 hasil; link lama tetap valid (backward compatible)</t>
   </si>
   <si>
+    <t xml:space="preserve">Selesai</t>
+  </si>
+  <si>
     <t xml:space="preserve">S-02</t>
   </si>
   <si>
@@ -119,6 +122,9 @@
   </si>
   <si>
     <t xml:space="preserve">App hidup di domain produksi dengan DB persisten; satu deploy penuh sukses dari repo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belum mulai</t>
   </si>
   <si>
     <t xml:space="preserve">S-04</t>
@@ -797,108 +803,104 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1182,544 +1184,575 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:K22"/>
+  <dimension ref="B1:K22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
   </cols>
   <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="K4" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="8" t="n">
+      <c r="I5" s="7" t="n">
         <v>0.25</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="K5" s="6"/>
+      <c r="K5" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="10" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="11" t="s">
+      <c r="E7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="K6" s="10"/>
-    </row>
-    <row r="7" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="6" t="s">
+      <c r="F7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" s="6"/>
-    </row>
-    <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="E8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="11" t="s">
+      <c r="E9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="K9" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="I8" s="12" t="n">
+    </row>
+    <row r="10" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="I11" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="J8" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="K8" s="10"/>
-    </row>
-    <row r="9" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="I9" s="8" t="n">
+      <c r="J11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="J9" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="K9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="11" t="s">
+      <c r="J13" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J16" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="I10" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="K10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="I11" s="8" t="n">
+      <c r="D17" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="I18" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="J11" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="K11" s="6"/>
-    </row>
-    <row r="12" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J12" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="K12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="I13" s="8" t="n">
+      <c r="J18" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="K18" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="I19" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="J13" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="K13" s="6"/>
-    </row>
-    <row r="14" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="I14" s="12" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="K14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="K15" s="6"/>
-    </row>
-    <row r="16" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="I16" s="12" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J16" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="K16" s="10"/>
-    </row>
-    <row r="17" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="I17" s="8" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="K17" s="6"/>
-    </row>
-    <row r="18" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="I18" s="12" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="K18" s="10"/>
-    </row>
-    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="I19" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="K19" s="6"/>
+      <c r="J19" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="I20" s="14" t="n">
+      <c r="B20" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="I20" s="13" t="n">
         <f aca="false">SUM(I5:I19)</f>
         <v>13.25</v>
       </c>
-      <c r="J20" s="13"/>
-      <c r="K20" s="13"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="3" t="s">
-        <v>109</v>
+      <c r="B22" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1749,400 +1782,401 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:G26"/>
+  <dimension ref="B1:G26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
   </cols>
   <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="B2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="3" t="s">
-        <v>111</v>
+      <c r="B3" s="2" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>117</v>
       </c>
+      <c r="F4" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="D5" s="16" t="s">
+      <c r="C5" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="F5" s="17" t="s">
+      <c r="E5" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G5" s="16" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="F6" s="20" t="s">
+      <c r="D6" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="G6" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="G6" s="19" t="s">
-        <v>121</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="F7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="G7" s="16" t="s">
-        <v>20</v>
+      <c r="D7" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="F8" s="20" t="s">
+      <c r="C8" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="G8" s="19" t="s">
-        <v>26</v>
+      <c r="D8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>26</v>
+      <c r="C9" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
+      <c r="B10" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="C11" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="F11" s="20" t="s">
+      <c r="C11" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="G11" s="19" t="s">
-        <v>26</v>
+      <c r="D11" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="F12" s="17" t="s">
+      <c r="C12" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="G12" s="16" t="s">
-        <v>121</v>
+      <c r="D12" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="C13" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="F13" s="20" t="s">
+      <c r="C13" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="G13" s="19" t="s">
-        <v>26</v>
+      <c r="D13" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="21" t="s">
-        <v>142</v>
-      </c>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
+      <c r="B14" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="15" t="n">
+      <c r="B15" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="C15" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="F15" s="17" t="s">
+      <c r="C15" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="G15" s="16" t="s">
-        <v>121</v>
+      <c r="D15" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="F16" s="20" t="s">
+      <c r="C16" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="D16" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>149</v>
       </c>
+      <c r="F16" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="15" t="n">
+      <c r="B17" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="C17" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="F17" s="17" t="s">
+      <c r="C17" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="G17" s="16" t="s">
-        <v>26</v>
+      <c r="D17" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
+      <c r="B18" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="C19" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="F19" s="20" t="s">
+      <c r="C19" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="G19" s="19" t="s">
-        <v>121</v>
+      <c r="D19" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="15" t="n">
+      <c r="B20" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="C20" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="F20" s="17" t="s">
+      <c r="C20" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="G20" s="16" t="s">
-        <v>74</v>
+      <c r="D20" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="18" t="n">
+      <c r="B21" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="C21" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="D21" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="F21" s="20" t="s">
+      <c r="C21" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="G21" s="19" t="s">
-        <v>121</v>
+      <c r="D21" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="15" t="n">
+      <c r="B22" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C22" s="16" t="s">
-        <v>160</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="F22" s="17" t="s">
-        <v>164</v>
-      </c>
-      <c r="G22" s="16" t="s">
-        <v>121</v>
+      <c r="C22" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="21" t="s">
-        <v>165</v>
-      </c>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
+      <c r="B23" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="3" t="s">
-        <v>166</v>
+      <c r="B25" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="3" t="s">
-        <v>167</v>
+      <c r="B26" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2168,162 +2202,163 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:D19"/>
+  <dimension ref="B1:D19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="40"/>
   </cols>
   <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>171</v>
       </c>
+      <c r="C4" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="22" t="s">
-        <v>172</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="B5" s="21" t="s">
         <v>174</v>
       </c>
+      <c r="C5" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="23" t="s">
-        <v>175</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="D6" s="11" t="s">
+      <c r="B6" s="22" t="s">
         <v>177</v>
       </c>
+      <c r="C6" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="22" t="s">
-        <v>178</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="B7" s="21" t="s">
         <v>180</v>
       </c>
+      <c r="C7" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="23" t="s">
-        <v>181</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D8" s="11" t="s">
+      <c r="B8" s="22" t="s">
         <v>183</v>
       </c>
+      <c r="C8" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="22" t="s">
-        <v>184</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="B9" s="21" t="s">
         <v>186</v>
       </c>
+      <c r="C9" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="23" t="s">
-        <v>187</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>188</v>
-      </c>
-      <c r="D10" s="11" t="s">
+      <c r="B10" s="22" t="s">
         <v>189</v>
       </c>
+      <c r="C10" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="B11" s="21" t="s">
         <v>192</v>
       </c>
+      <c r="C11" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="24" t="s">
-        <v>193</v>
-      </c>
-      <c r="D12" s="24" t="s">
-        <v>194</v>
+      <c r="C12" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="25" t="s">
-        <v>195</v>
+      <c r="B14" s="24" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>198</v>
       </c>
+      <c r="C15" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="22" t="s">
-        <v>199</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="D16" s="7" t="s">
+      <c r="B16" s="21" t="s">
         <v>201</v>
       </c>
+      <c r="C16" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="23" t="s">
-        <v>202</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>203</v>
-      </c>
-      <c r="D17" s="11" t="s">
+      <c r="B17" s="22" t="s">
         <v>204</v>
       </c>
+      <c r="C17" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="3" t="s">
-        <v>205</v>
+      <c r="B19" s="2" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>